<commit_message>
Refresh solar module & cell data with latest NISE portal figures
Re-pulled current portal values; keeps the same calendar-year layout.
Minor June 2026 revision (Bluebird Solar 0.14 -> 0.16); module and cell
TOTALs continue to reconcile to the portal grand totals.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BDTseMcVZsdeEbJn1jNXqJ
</commit_message>
<xml_diff>
--- a/Solar_modules_and_cells.xlsx
+++ b/Solar_modules_and_cells.xlsx
@@ -2458,7 +2458,7 @@
         <v>0.13</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="13">
@@ -6301,7 +6301,7 @@
         <v>15.58</v>
       </c>
       <c r="S75" s="4" t="n">
-        <v>26.7</v>
+        <v>26.68</v>
       </c>
     </row>
     <row r="76">

</xml_diff>

<commit_message>
Add July 2026 column and refresh all months from NISE DCR portal
Append July 2026 to both sheets (same calendar-year layout) and refresh
every prior month to the portal's current values; late DCR filings had
pushed several months up materially since the last pull (e.g. module
Jun 2026 2124 -> 2370 MW).

- July 2026: modules 1867.8 MW, cells 1014.8 MW.
- Module Others row recomputed so each month's TOTAL equals the portal
  grand total (verified exact across all months); small new registrants
  (Reliance, Premier Energies International, Veda, Solex, Asote) fold in.
- Handled portal rename Contendre Greenergy Private Limited ->
  Contendre Greenergy Limited so its row refreshes.
- Extended TOTAL, Key-Players summary, and FY YTD sections to July.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BDTseMcVZsdeEbJn1jNXqJ
</commit_message>
<xml_diff>
--- a/Solar_modules_and_cells.xlsx
+++ b/Solar_modules_and_cells.xlsx
@@ -1777,13 +1777,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:S120"/>
+  <dimension ref="A2:T120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="51.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="10.7109375" customWidth="1" min="2" max="18"/>
     <col width="13" customWidth="1" min="18" max="18"/>
     <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1817,7 +1818,8 @@
       <c r="P2" s="35" t="n"/>
       <c r="Q2" s="35" t="n"/>
       <c r="R2" s="35" t="n"/>
-      <c r="S2" s="36" t="n"/>
+      <c r="S2" s="35" t="n"/>
+      <c r="T2" s="36" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="37" t="n"/>
@@ -1911,6 +1913,11 @@
           <t>Jun</t>
         </is>
       </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1972,6 +1979,9 @@
       <c r="S4" s="4" t="n">
         <v>2.35</v>
       </c>
+      <c r="T4" s="4" t="n">
+        <v>4.25</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2033,6 +2043,9 @@
       <c r="S5" s="4" t="n">
         <v>6.16</v>
       </c>
+      <c r="T5" s="4" t="n">
+        <v>5.04</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2092,7 +2105,10 @@
         <v>14.98</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>14.15</v>
+        <v>14.16</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>21.59</v>
       </c>
     </row>
     <row r="7">
@@ -2153,7 +2169,10 @@
         <v>0.13</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
+      </c>
+      <c r="T7" s="4" t="n">
+        <v>0.12</v>
       </c>
     </row>
     <row r="8">
@@ -2211,10 +2230,13 @@
         <v>1.37</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>9.380000000000001</v>
+        <v>10.18</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0</v>
+        <v>1.05</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>6.03</v>
       </c>
     </row>
     <row r="9">
@@ -2275,7 +2297,10 @@
         <v>44.72</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>59.42</v>
+        <v>60.77</v>
+      </c>
+      <c r="T9" s="4" t="n">
+        <v>56.51</v>
       </c>
     </row>
     <row r="10">
@@ -2333,10 +2358,13 @@
         <v>1.97</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>4.81</v>
+        <v>4.93</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>4.25</v>
+        <v>5.56</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>3.39</v>
       </c>
     </row>
     <row r="11">
@@ -2346,13 +2374,13 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>11.83</v>
+        <v>12.36</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>11.27</v>
+        <v>12.31</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>13.46</v>
+        <v>14</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>6.13</v>
@@ -2367,10 +2395,10 @@
         <v>5.74</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>4.39</v>
+        <v>4.23</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>7.11</v>
+        <v>7.52</v>
       </c>
       <c r="K11" s="4" t="n">
         <v>4.49</v>
@@ -2379,7 +2407,7 @@
         <v>12.52</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>10.53</v>
+        <v>10.76</v>
       </c>
       <c r="N11" s="4" t="n">
         <v>9.369999999999999</v>
@@ -2391,13 +2419,16 @@
         <v>6.73</v>
       </c>
       <c r="Q11" s="4" t="n">
-        <v>9.18</v>
+        <v>9.17</v>
       </c>
       <c r="R11" s="4" t="n">
-        <v>16.17</v>
+        <v>16.18</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>23.42</v>
+        <v>24.02</v>
+      </c>
+      <c r="T11" s="4" t="n">
+        <v>22.13</v>
       </c>
     </row>
     <row r="12">
@@ -2458,7 +2489,10 @@
         <v>0.13</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.16</v>
+        <v>0.62</v>
+      </c>
+      <c r="T12" s="4" t="n">
+        <v>0.13</v>
       </c>
     </row>
     <row r="13">
@@ -2471,55 +2505,58 @@
         <v>3.13</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>3.85</v>
+        <v>3.84</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>5.71</v>
+        <v>5.59</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>4.32</v>
+        <v>4.2</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>12.49</v>
+        <v>12.39</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>11.52</v>
+        <v>11.4</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>10.39</v>
+        <v>10.27</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>5.95</v>
+        <v>5.7</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>3.02</v>
+        <v>2.73</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>2.19</v>
+        <v>2.05</v>
       </c>
       <c r="L13" s="4" t="n">
-        <v>8.41</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>5.63</v>
+        <v>5.11</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>12.21</v>
+        <v>11.15</v>
       </c>
       <c r="O13" s="4" t="n">
-        <v>12.31</v>
+        <v>12.19</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>13.38</v>
+        <v>13.17</v>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>5.9</v>
+        <v>5.24</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>10.11</v>
+        <v>9.59</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>6.08</v>
+        <v>5.74</v>
+      </c>
+      <c r="T13" s="4" t="n">
+        <v>8.460000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -2571,7 +2608,7 @@
         <v>0.31</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>0.27</v>
+        <v>0.52</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>0</v>
@@ -2580,7 +2617,10 @@
         <v>0.25</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0</v>
+        <v>0.06</v>
+      </c>
+      <c r="T14" s="4" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="15">
@@ -2632,10 +2672,10 @@
         <v>0.46</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>1.72</v>
+        <v>1.83</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="R15" s="4" t="n">
         <v>0.44</v>
@@ -2643,6 +2683,9 @@
       <c r="S15" s="4" t="n">
         <v>3.63</v>
       </c>
+      <c r="T15" s="4" t="n">
+        <v>0.44</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2702,7 +2745,10 @@
         <v>9.52</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>28.7</v>
+        <v>30.43</v>
+      </c>
+      <c r="T16" s="4" t="n">
+        <v>31.71</v>
       </c>
     </row>
     <row r="17">
@@ -2765,6 +2811,9 @@
       <c r="S17" s="4" t="n">
         <v>2.91</v>
       </c>
+      <c r="T17" s="4" t="n">
+        <v>2.32</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -2824,7 +2873,10 @@
         <v>2.81</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>2.89</v>
+        <v>3.65</v>
+      </c>
+      <c r="T18" s="4" t="n">
+        <v>1.88</v>
       </c>
     </row>
     <row r="19">
@@ -2887,6 +2939,9 @@
       <c r="S19" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="T19" s="4" t="n">
+        <v>21.27</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -2913,7 +2968,7 @@
         <v>96.98</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>120.62</v>
+        <v>119.45</v>
       </c>
       <c r="I20" s="4" t="n">
         <v>69.79000000000001</v>
@@ -2922,7 +2977,7 @@
         <v>18.63</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>44.9</v>
+        <v>44.85</v>
       </c>
       <c r="L20" s="4" t="n">
         <v>20.36</v>
@@ -2943,10 +2998,13 @@
         <v>24.87</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>66.69</v>
+        <v>66.7</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>121.75</v>
+        <v>121.9</v>
+      </c>
+      <c r="T20" s="4" t="n">
+        <v>52.36</v>
       </c>
     </row>
     <row r="21">
@@ -2995,19 +3053,22 @@
         <v>244.78</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>182.62</v>
+        <v>182.66</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>319.99</v>
+        <v>323.05</v>
       </c>
       <c r="Q21" s="4" t="n">
-        <v>16.27</v>
+        <v>25.25</v>
       </c>
       <c r="R21" s="4" t="n">
-        <v>17.36</v>
+        <v>18.13</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>4.56</v>
+        <v>8.640000000000001</v>
+      </c>
+      <c r="T21" s="4" t="n">
+        <v>46.57</v>
       </c>
     </row>
     <row r="22">
@@ -3065,10 +3126,13 @@
         <v>49.07</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>73.55</v>
+        <v>73.72</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>88.05</v>
+        <v>90.83</v>
+      </c>
+      <c r="T22" s="4" t="n">
+        <v>74.95999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -3131,6 +3195,9 @@
       <c r="S23" s="4" t="n">
         <v>12.32</v>
       </c>
+      <c r="T23" s="4" t="n">
+        <v>17.94</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -3187,10 +3254,13 @@
         <v>5.78</v>
       </c>
       <c r="R24" s="4" t="n">
-        <v>8.130000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>20.7</v>
+        <v>22.89</v>
+      </c>
+      <c r="T24" s="4" t="n">
+        <v>10.33</v>
       </c>
     </row>
     <row r="25">
@@ -3239,19 +3309,22 @@
         <v>0.71</v>
       </c>
       <c r="O25" s="4" t="n">
-        <v>0.37</v>
+        <v>0.79</v>
       </c>
       <c r="P25" s="4" t="n">
         <v>14.59</v>
       </c>
       <c r="Q25" s="4" t="n">
-        <v>0.5</v>
+        <v>4.14</v>
       </c>
       <c r="R25" s="4" t="n">
-        <v>1.44</v>
+        <v>1.52</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>0.46</v>
+        <v>1.98</v>
+      </c>
+      <c r="T25" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -3303,16 +3376,19 @@
         <v>1.11</v>
       </c>
       <c r="P26" s="4" t="n">
-        <v>9.76</v>
+        <v>4.79</v>
       </c>
       <c r="Q26" s="4" t="n">
-        <v>3.35</v>
+        <v>5.59</v>
       </c>
       <c r="R26" s="4" t="n">
-        <v>16.53</v>
+        <v>16.78</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>3.25</v>
+        <v>9.17</v>
+      </c>
+      <c r="T26" s="4" t="n">
+        <v>7.65</v>
       </c>
     </row>
     <row r="27">
@@ -3361,19 +3437,22 @@
         <v>1.82</v>
       </c>
       <c r="O27" s="4" t="n">
-        <v>3.64</v>
+        <v>3.65</v>
       </c>
       <c r="P27" s="4" t="n">
         <v>3.91</v>
       </c>
       <c r="Q27" s="4" t="n">
-        <v>1.15</v>
+        <v>1.17</v>
       </c>
       <c r="R27" s="4" t="n">
-        <v>5.67</v>
+        <v>5.88</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>6.15</v>
+        <v>7.07</v>
+      </c>
+      <c r="T27" s="4" t="n">
+        <v>7.73</v>
       </c>
     </row>
     <row r="28">
@@ -3434,7 +3513,10 @@
         <v>7.88</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>13.14</v>
+        <v>13.25</v>
+      </c>
+      <c r="T28" s="4" t="n">
+        <v>13.35</v>
       </c>
     </row>
     <row r="29">
@@ -3483,19 +3565,22 @@
         <v>30.64</v>
       </c>
       <c r="O29" s="4" t="n">
-        <v>47.29</v>
+        <v>47.28</v>
       </c>
       <c r="P29" s="4" t="n">
         <v>59.91</v>
       </c>
       <c r="Q29" s="4" t="n">
-        <v>28.37</v>
+        <v>28.28</v>
       </c>
       <c r="R29" s="4" t="n">
-        <v>33.02</v>
+        <v>33.03</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>28.78</v>
+        <v>31.7</v>
+      </c>
+      <c r="T29" s="4" t="n">
+        <v>42.85</v>
       </c>
     </row>
     <row r="30">
@@ -3544,19 +3629,22 @@
         <v>10.66</v>
       </c>
       <c r="O30" s="4" t="n">
-        <v>10.21</v>
+        <v>6.9</v>
       </c>
       <c r="P30" s="4" t="n">
-        <v>33.41</v>
+        <v>27.61</v>
       </c>
       <c r="Q30" s="4" t="n">
-        <v>15.11</v>
+        <v>13.04</v>
       </c>
       <c r="R30" s="4" t="n">
         <v>47.71</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>51.21</v>
+        <v>54.41</v>
+      </c>
+      <c r="T30" s="4" t="n">
+        <v>29.71</v>
       </c>
     </row>
     <row r="31">
@@ -3599,10 +3687,10 @@
         <v>7.93</v>
       </c>
       <c r="M31" s="4" t="n">
-        <v>8.83</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="N31" s="4" t="n">
-        <v>13.42</v>
+        <v>13.28</v>
       </c>
       <c r="O31" s="4" t="n">
         <v>14.47</v>
@@ -3614,11 +3702,14 @@
         <v>5.99</v>
       </c>
       <c r="R31" s="4" t="n">
-        <v>13.73</v>
+        <v>13.62</v>
       </c>
       <c r="S31" s="4" t="n">
         <v>13.32</v>
       </c>
+      <c r="T31" s="4" t="n">
+        <v>12.41</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -3651,7 +3742,7 @@
         <v>0.58</v>
       </c>
       <c r="J32" s="4" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="K32" s="4" t="n">
         <v>0.8</v>
@@ -3660,7 +3751,7 @@
         <v>0.91</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>0.71</v>
+        <v>0.72</v>
       </c>
       <c r="N32" s="4" t="n">
         <v>0.44</v>
@@ -3678,7 +3769,10 @@
         <v>0.45</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.34</v>
+        <v>0.46</v>
+      </c>
+      <c r="T32" s="4" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="33">
@@ -3741,6 +3835,9 @@
       <c r="S33" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="T33" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -3782,7 +3879,7 @@
         <v>1.59</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>5.85</v>
+        <v>5.95</v>
       </c>
       <c r="N34" s="4" t="n">
         <v>5.05</v>
@@ -3794,13 +3891,16 @@
         <v>13.5</v>
       </c>
       <c r="Q34" s="4" t="n">
-        <v>7.87</v>
+        <v>10.73</v>
       </c>
       <c r="R34" s="4" t="n">
         <v>3.09</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>2.75</v>
+        <v>3.51</v>
+      </c>
+      <c r="T34" s="4" t="n">
+        <v>4.19</v>
       </c>
     </row>
     <row r="35">
@@ -3852,7 +3952,7 @@
         <v>4.02</v>
       </c>
       <c r="P35" s="4" t="n">
-        <v>6.28</v>
+        <v>6.29</v>
       </c>
       <c r="Q35" s="4" t="n">
         <v>0.02</v>
@@ -3863,6 +3963,9 @@
       <c r="S35" s="4" t="n">
         <v>3.44</v>
       </c>
+      <c r="T35" s="4" t="n">
+        <v>2.16</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -3924,6 +4027,9 @@
       <c r="S36" s="4" t="n">
         <v>5.07</v>
       </c>
+      <c r="T36" s="4" t="n">
+        <v>12.1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -3974,16 +4080,19 @@
         <v>1.21</v>
       </c>
       <c r="P37" s="4" t="n">
-        <v>28.85</v>
+        <v>45.77</v>
       </c>
       <c r="Q37" s="4" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="R37" s="4" t="n">
-        <v>1.65</v>
+        <v>3.21</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>3.02</v>
+        <v>6.02</v>
+      </c>
+      <c r="T37" s="4" t="n">
+        <v>5.62</v>
       </c>
     </row>
     <row r="38">
@@ -4046,6 +4155,9 @@
       <c r="S38" s="4" t="n">
         <v>9.65</v>
       </c>
+      <c r="T38" s="4" t="n">
+        <v>2.05</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -4090,10 +4202,10 @@
         <v>5.62</v>
       </c>
       <c r="N39" s="4" t="n">
-        <v>4.27</v>
+        <v>4.29</v>
       </c>
       <c r="O39" s="4" t="n">
-        <v>4.46</v>
+        <v>4.49</v>
       </c>
       <c r="P39" s="4" t="n">
         <v>4.25</v>
@@ -4105,7 +4217,10 @@
         <v>19.14</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>14.67</v>
+        <v>15.74</v>
+      </c>
+      <c r="T39" s="4" t="n">
+        <v>14.38</v>
       </c>
     </row>
     <row r="40">
@@ -4163,10 +4278,13 @@
         <v>38.34</v>
       </c>
       <c r="R40" s="4" t="n">
-        <v>53.18</v>
+        <v>53.2</v>
       </c>
       <c r="S40" s="4" t="n">
-        <v>70.16</v>
+        <v>79.66</v>
+      </c>
+      <c r="T40" s="4" t="n">
+        <v>35.95</v>
       </c>
     </row>
     <row r="41">
@@ -4215,7 +4333,7 @@
         <v>147.98</v>
       </c>
       <c r="O41" s="4" t="n">
-        <v>130.46</v>
+        <v>130.54</v>
       </c>
       <c r="P41" s="4" t="n">
         <v>178.68</v>
@@ -4224,10 +4342,13 @@
         <v>161.71</v>
       </c>
       <c r="R41" s="4" t="n">
-        <v>136.93</v>
+        <v>137.26</v>
       </c>
       <c r="S41" s="4" t="n">
-        <v>119.15</v>
+        <v>174.05</v>
+      </c>
+      <c r="T41" s="4" t="n">
+        <v>120.08</v>
       </c>
     </row>
     <row r="42">
@@ -4285,10 +4406,13 @@
         <v>119.68</v>
       </c>
       <c r="R42" s="4" t="n">
-        <v>183.93</v>
+        <v>183.92</v>
       </c>
       <c r="S42" s="4" t="n">
-        <v>92.75</v>
+        <v>149.54</v>
+      </c>
+      <c r="T42" s="4" t="n">
+        <v>99.20999999999999</v>
       </c>
     </row>
     <row r="43">
@@ -4328,7 +4452,7 @@
         <v>3.99</v>
       </c>
       <c r="L43" s="4" t="n">
-        <v>8.85</v>
+        <v>8.48</v>
       </c>
       <c r="M43" s="4" t="n">
         <v>5.04</v>
@@ -4349,7 +4473,10 @@
         <v>6.08</v>
       </c>
       <c r="S43" s="4" t="n">
-        <v>3.25</v>
+        <v>3.28</v>
+      </c>
+      <c r="T43" s="4" t="n">
+        <v>5.12</v>
       </c>
     </row>
     <row r="44">
@@ -4412,6 +4539,9 @@
       <c r="S44" s="4" t="n">
         <v>0.23</v>
       </c>
+      <c r="T44" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -4435,16 +4565,16 @@
         <v>7.18</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>7.75</v>
+        <v>8.65</v>
       </c>
       <c r="H45" s="4" t="n">
-        <v>8.49</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="I45" s="4" t="n">
-        <v>8.4</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="J45" s="4" t="n">
-        <v>5.77</v>
+        <v>6.15</v>
       </c>
       <c r="K45" s="4" t="n">
         <v>4.27</v>
@@ -4471,7 +4601,10 @@
         <v>5.81</v>
       </c>
       <c r="S45" s="4" t="n">
-        <v>10.25</v>
+        <v>11.48</v>
+      </c>
+      <c r="T45" s="4" t="n">
+        <v>7.75</v>
       </c>
     </row>
     <row r="46">
@@ -4532,7 +4665,10 @@
         <v>31.3</v>
       </c>
       <c r="S46" s="4" t="n">
-        <v>33.28</v>
+        <v>33.83</v>
+      </c>
+      <c r="T46" s="4" t="n">
+        <v>20.91</v>
       </c>
     </row>
     <row r="47">
@@ -4590,10 +4726,13 @@
         <v>5.93</v>
       </c>
       <c r="R47" s="4" t="n">
-        <v>7.16</v>
+        <v>7.12</v>
       </c>
       <c r="S47" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>9.51</v>
+      </c>
+      <c r="T47" s="4" t="n">
+        <v>7.5</v>
       </c>
     </row>
     <row r="48">
@@ -4654,7 +4793,10 @@
         <v>1.02</v>
       </c>
       <c r="S48" s="4" t="n">
-        <v>1.24</v>
+        <v>1.31</v>
+      </c>
+      <c r="T48" s="4" t="n">
+        <v>0.48</v>
       </c>
     </row>
     <row r="49">
@@ -4715,7 +4857,10 @@
         <v>2.24</v>
       </c>
       <c r="S49" s="4" t="n">
-        <v>1.76</v>
+        <v>2.24</v>
+      </c>
+      <c r="T49" s="4" t="n">
+        <v>0.98</v>
       </c>
     </row>
     <row r="50">
@@ -4770,13 +4915,16 @@
         <v>136.58</v>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>53.44</v>
+        <v>53.51</v>
       </c>
       <c r="R50" s="4" t="n">
         <v>82.75</v>
       </c>
       <c r="S50" s="4" t="n">
-        <v>70.64</v>
+        <v>86.54000000000001</v>
+      </c>
+      <c r="T50" s="4" t="n">
+        <v>102.33</v>
       </c>
     </row>
     <row r="51">
@@ -4822,7 +4970,7 @@
         <v>40.33</v>
       </c>
       <c r="N51" s="4" t="n">
-        <v>36.08</v>
+        <v>36.1</v>
       </c>
       <c r="O51" s="4" t="n">
         <v>71.84999999999999</v>
@@ -4837,7 +4985,10 @@
         <v>97.22</v>
       </c>
       <c r="S51" s="4" t="n">
-        <v>174</v>
+        <v>174.51</v>
+      </c>
+      <c r="T51" s="4" t="n">
+        <v>96.03</v>
       </c>
     </row>
     <row r="52">
@@ -4892,7 +5043,7 @@
         <v>6.2</v>
       </c>
       <c r="Q52" s="4" t="n">
-        <v>1.86</v>
+        <v>1.87</v>
       </c>
       <c r="R52" s="4" t="n">
         <v>3.46</v>
@@ -4900,6 +5051,9 @@
       <c r="S52" s="4" t="n">
         <v>5.02</v>
       </c>
+      <c r="T52" s="4" t="n">
+        <v>4.4</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -4961,6 +5115,9 @@
       <c r="S53" s="4" t="n">
         <v>3.54</v>
       </c>
+      <c r="T53" s="4" t="n">
+        <v>1.75</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -4969,13 +5126,13 @@
         </is>
       </c>
       <c r="B54" s="4" t="n">
-        <v>14.41</v>
+        <v>13.87</v>
       </c>
       <c r="C54" s="4" t="n">
-        <v>8.140000000000001</v>
+        <v>7.84</v>
       </c>
       <c r="D54" s="4" t="n">
-        <v>9.35</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="E54" s="4" t="n">
         <v>6.06</v>
@@ -5020,7 +5177,10 @@
         <v>43.21</v>
       </c>
       <c r="S54" s="4" t="n">
-        <v>63.21</v>
+        <v>63.9</v>
+      </c>
+      <c r="T54" s="4" t="n">
+        <v>55.03</v>
       </c>
     </row>
     <row r="55">
@@ -5081,7 +5241,10 @@
         <v>20.51</v>
       </c>
       <c r="S55" s="4" t="n">
-        <v>15.26</v>
+        <v>15.33</v>
+      </c>
+      <c r="T55" s="4" t="n">
+        <v>19.44</v>
       </c>
     </row>
     <row r="56">
@@ -5097,10 +5260,10 @@
         <v>129.5</v>
       </c>
       <c r="D56" s="4" t="n">
-        <v>123.21</v>
+        <v>122.02</v>
       </c>
       <c r="E56" s="4" t="n">
-        <v>88.76000000000001</v>
+        <v>87.5</v>
       </c>
       <c r="F56" s="4" t="n">
         <v>99.59</v>
@@ -5109,40 +5272,43 @@
         <v>58.06</v>
       </c>
       <c r="H56" s="4" t="n">
-        <v>58.94</v>
+        <v>53.29</v>
       </c>
       <c r="I56" s="4" t="n">
-        <v>34.1</v>
+        <v>28.5</v>
       </c>
       <c r="J56" s="4" t="n">
         <v>35.48</v>
       </c>
       <c r="K56" s="4" t="n">
-        <v>41.33</v>
+        <v>36.39</v>
       </c>
       <c r="L56" s="4" t="n">
-        <v>21.6</v>
+        <v>19.64</v>
       </c>
       <c r="M56" s="4" t="n">
-        <v>31.73</v>
+        <v>24.11</v>
       </c>
       <c r="N56" s="4" t="n">
-        <v>62.81</v>
+        <v>55.75</v>
       </c>
       <c r="O56" s="4" t="n">
-        <v>71.56999999999999</v>
+        <v>66.86</v>
       </c>
       <c r="P56" s="4" t="n">
-        <v>77.11</v>
+        <v>72.01000000000001</v>
       </c>
       <c r="Q56" s="4" t="n">
-        <v>68.75</v>
+        <v>59</v>
       </c>
       <c r="R56" s="4" t="n">
-        <v>155.29</v>
+        <v>137.53</v>
       </c>
       <c r="S56" s="4" t="n">
-        <v>131.81</v>
+        <v>113.88</v>
+      </c>
+      <c r="T56" s="4" t="n">
+        <v>77.51000000000001</v>
       </c>
     </row>
     <row r="57">
@@ -5164,7 +5330,7 @@
         <v>0</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>0</v>
@@ -5203,7 +5369,10 @@
         <v>8.960000000000001</v>
       </c>
       <c r="S57" s="4" t="n">
-        <v>3.79</v>
+        <v>10.96</v>
+      </c>
+      <c r="T57" s="4" t="n">
+        <v>3.34</v>
       </c>
     </row>
     <row r="58">
@@ -5261,11 +5430,14 @@
         <v>1.22</v>
       </c>
       <c r="R58" s="4" t="n">
-        <v>2.98</v>
+        <v>2.99</v>
       </c>
       <c r="S58" s="4" t="n">
         <v>3.71</v>
       </c>
+      <c r="T58" s="4" t="n">
+        <v>4.48</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -5283,10 +5455,10 @@
         <v>3.71</v>
       </c>
       <c r="E59" s="4" t="n">
-        <v>1.99</v>
+        <v>2.11</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>6.87</v>
+        <v>6.94</v>
       </c>
       <c r="G59" s="4" t="n">
         <v>6.15</v>
@@ -5313,19 +5485,22 @@
         <v>2.03</v>
       </c>
       <c r="O59" s="4" t="n">
-        <v>2.32</v>
+        <v>2.31</v>
       </c>
       <c r="P59" s="4" t="n">
         <v>1.37</v>
       </c>
       <c r="Q59" s="4" t="n">
-        <v>0.28</v>
+        <v>0.19</v>
       </c>
       <c r="R59" s="4" t="n">
         <v>0.02</v>
       </c>
       <c r="S59" s="4" t="n">
-        <v>2.9</v>
+        <v>3.87</v>
+      </c>
+      <c r="T59" s="4" t="n">
+        <v>4.95</v>
       </c>
     </row>
     <row r="60">
@@ -5383,10 +5558,13 @@
         <v>0.06</v>
       </c>
       <c r="R60" s="4" t="n">
-        <v>8.369999999999999</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="S60" s="4" t="n">
-        <v>4.04</v>
+        <v>6.67</v>
+      </c>
+      <c r="T60" s="4" t="n">
+        <v>2.13</v>
       </c>
     </row>
     <row r="61">
@@ -5449,6 +5627,9 @@
       <c r="S61" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="T61" s="4" t="n">
+        <v>0.38</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -5496,7 +5677,7 @@
         <v>1.06</v>
       </c>
       <c r="O62" s="4" t="n">
-        <v>2.07</v>
+        <v>2.08</v>
       </c>
       <c r="P62" s="4" t="n">
         <v>4.21</v>
@@ -5505,10 +5686,13 @@
         <v>1.37</v>
       </c>
       <c r="R62" s="4" t="n">
-        <v>2.27</v>
+        <v>2.48</v>
       </c>
       <c r="S62" s="4" t="n">
-        <v>4.42</v>
+        <v>4.45</v>
+      </c>
+      <c r="T62" s="4" t="n">
+        <v>3.87</v>
       </c>
     </row>
     <row r="63">
@@ -5569,7 +5753,10 @@
         <v>2.14</v>
       </c>
       <c r="S63" s="4" t="n">
-        <v>3.25</v>
+        <v>3.3</v>
+      </c>
+      <c r="T63" s="4" t="n">
+        <v>4.2</v>
       </c>
     </row>
     <row r="64">
@@ -5630,7 +5817,10 @@
         <v>0.4</v>
       </c>
       <c r="S64" s="4" t="n">
-        <v>1.61</v>
+        <v>1.76</v>
+      </c>
+      <c r="T64" s="4" t="n">
+        <v>4.79</v>
       </c>
     </row>
     <row r="65">
@@ -5682,16 +5872,19 @@
         <v>12.52</v>
       </c>
       <c r="P65" s="4" t="n">
-        <v>9.49</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="Q65" s="4" t="n">
-        <v>0.85</v>
+        <v>1.38</v>
       </c>
       <c r="R65" s="4" t="n">
-        <v>5.84</v>
+        <v>15.32</v>
       </c>
       <c r="S65" s="4" t="n">
-        <v>5.08</v>
+        <v>7.44</v>
+      </c>
+      <c r="T65" s="4" t="n">
+        <v>3.83</v>
       </c>
     </row>
     <row r="66">
@@ -5710,10 +5903,10 @@
         <v>5.16</v>
       </c>
       <c r="E66" s="4" t="n">
-        <v>3.1</v>
+        <v>2.57</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>3.76</v>
+        <v>2.95</v>
       </c>
       <c r="G66" s="4" t="n">
         <v>3.47</v>
@@ -5734,7 +5927,7 @@
         <v>3.13</v>
       </c>
       <c r="M66" s="4" t="n">
-        <v>3.42</v>
+        <v>3.43</v>
       </c>
       <c r="N66" s="4" t="n">
         <v>4.5</v>
@@ -5743,16 +5936,19 @@
         <v>4.96</v>
       </c>
       <c r="P66" s="4" t="n">
-        <v>4.9</v>
+        <v>5.55</v>
       </c>
       <c r="Q66" s="4" t="n">
-        <v>2.86</v>
+        <v>1.22</v>
       </c>
       <c r="R66" s="4" t="n">
-        <v>2.77</v>
+        <v>2.28</v>
       </c>
       <c r="S66" s="4" t="n">
-        <v>3.43</v>
+        <v>3.6</v>
+      </c>
+      <c r="T66" s="4" t="n">
+        <v>3.33</v>
       </c>
     </row>
     <row r="67">
@@ -5780,31 +5976,31 @@
         <v>0.54</v>
       </c>
       <c r="H67" s="4" t="n">
-        <v>0.74</v>
+        <v>0.98</v>
       </c>
       <c r="I67" s="4" t="n">
-        <v>0.78</v>
+        <v>0.79</v>
       </c>
       <c r="J67" s="4" t="n">
         <v>0.97</v>
       </c>
       <c r="K67" s="4" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="L67" s="4" t="n">
         <v>1.26</v>
       </c>
       <c r="M67" s="4" t="n">
-        <v>1.11</v>
+        <v>1.12</v>
       </c>
       <c r="N67" s="4" t="n">
         <v>0.8</v>
       </c>
       <c r="O67" s="4" t="n">
-        <v>2.55</v>
+        <v>2.58</v>
       </c>
       <c r="P67" s="4" t="n">
-        <v>2.27</v>
+        <v>2.31</v>
       </c>
       <c r="Q67" s="4" t="n">
         <v>0.6899999999999999</v>
@@ -5813,7 +6009,10 @@
         <v>0.93</v>
       </c>
       <c r="S67" s="4" t="n">
-        <v>1.94</v>
+        <v>2.68</v>
+      </c>
+      <c r="T67" s="4" t="n">
+        <v>0.27</v>
       </c>
     </row>
     <row r="68">
@@ -5844,7 +6043,7 @@
         <v>256.3</v>
       </c>
       <c r="I68" s="4" t="n">
-        <v>267.6</v>
+        <v>267.62</v>
       </c>
       <c r="J68" s="4" t="n">
         <v>557.0599999999999</v>
@@ -5853,28 +6052,31 @@
         <v>251.78</v>
       </c>
       <c r="L68" s="4" t="n">
-        <v>270.63</v>
+        <v>270.65</v>
       </c>
       <c r="M68" s="4" t="n">
-        <v>169.91</v>
+        <v>169.92</v>
       </c>
       <c r="N68" s="4" t="n">
-        <v>88.14</v>
+        <v>88.15000000000001</v>
       </c>
       <c r="O68" s="4" t="n">
-        <v>96.17</v>
+        <v>96.18000000000001</v>
       </c>
       <c r="P68" s="4" t="n">
-        <v>121.16</v>
+        <v>121.19</v>
       </c>
       <c r="Q68" s="4" t="n">
         <v>84.09999999999999</v>
       </c>
       <c r="R68" s="4" t="n">
-        <v>123.84</v>
+        <v>123.92</v>
       </c>
       <c r="S68" s="4" t="n">
-        <v>156.92</v>
+        <v>158.94</v>
+      </c>
+      <c r="T68" s="4" t="n">
+        <v>152.82</v>
       </c>
     </row>
     <row r="69">
@@ -5937,6 +6139,9 @@
       <c r="S69" s="4" t="n">
         <v>1.55</v>
       </c>
+      <c r="T69" s="4" t="n">
+        <v>1.62</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
@@ -5990,13 +6195,16 @@
         <v>5.44</v>
       </c>
       <c r="Q70" s="4" t="n">
-        <v>3.09</v>
+        <v>3.17</v>
       </c>
       <c r="R70" s="4" t="n">
         <v>4.56</v>
       </c>
       <c r="S70" s="4" t="n">
-        <v>8.5</v>
+        <v>8.59</v>
+      </c>
+      <c r="T70" s="4" t="n">
+        <v>11.13</v>
       </c>
     </row>
     <row r="71">
@@ -6054,10 +6262,13 @@
         <v>0.65</v>
       </c>
       <c r="R71" s="4" t="n">
-        <v>1.04</v>
+        <v>1.4</v>
       </c>
       <c r="S71" s="4" t="n">
-        <v>2.17</v>
+        <v>2.21</v>
+      </c>
+      <c r="T71" s="4" t="n">
+        <v>1.42</v>
       </c>
     </row>
     <row r="72">
@@ -6118,7 +6329,10 @@
         <v>18.74</v>
       </c>
       <c r="S72" s="4" t="n">
-        <v>43.49</v>
+        <v>50.75</v>
+      </c>
+      <c r="T72" s="4" t="n">
+        <v>22.06</v>
       </c>
     </row>
     <row r="73">
@@ -6155,7 +6369,7 @@
         <v>61.3</v>
       </c>
       <c r="K73" s="4" t="n">
-        <v>90.19</v>
+        <v>90.2</v>
       </c>
       <c r="L73" s="4" t="n">
         <v>144.08</v>
@@ -6173,13 +6387,16 @@
         <v>245.68</v>
       </c>
       <c r="Q73" s="4" t="n">
-        <v>229.75</v>
+        <v>229.77</v>
       </c>
       <c r="R73" s="4" t="n">
-        <v>281.25</v>
+        <v>281.29</v>
       </c>
       <c r="S73" s="4" t="n">
-        <v>463.13</v>
+        <v>484.5</v>
+      </c>
+      <c r="T73" s="4" t="n">
+        <v>385.45</v>
       </c>
     </row>
     <row r="74">
@@ -6225,7 +6442,7 @@
         <v>14.81</v>
       </c>
       <c r="N74" s="4" t="n">
-        <v>9.67</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="O74" s="4" t="n">
         <v>14.34</v>
@@ -6237,10 +6454,13 @@
         <v>9.960000000000001</v>
       </c>
       <c r="R74" s="4" t="n">
-        <v>35.61</v>
+        <v>35.11</v>
       </c>
       <c r="S74" s="4" t="n">
-        <v>25.53</v>
+        <v>28.46</v>
+      </c>
+      <c r="T74" s="4" t="n">
+        <v>5.35</v>
       </c>
     </row>
     <row r="75">
@@ -6250,58 +6470,61 @@
         </is>
       </c>
       <c r="B75" s="4" t="n">
-        <v>5.62</v>
+        <v>6.65</v>
       </c>
       <c r="C75" s="4" t="n">
-        <v>15.81</v>
+        <v>16.8</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>11.56</v>
+        <v>13.61</v>
       </c>
       <c r="E75" s="4" t="n">
-        <v>7.98</v>
+        <v>9.26</v>
       </c>
       <c r="F75" s="4" t="n">
-        <v>10.57</v>
+        <v>12.23</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>18.32</v>
+        <v>19.74</v>
       </c>
       <c r="H75" s="4" t="n">
-        <v>15.85</v>
+        <v>18.8</v>
       </c>
       <c r="I75" s="4" t="n">
-        <v>8.779999999999999</v>
+        <v>14.16</v>
       </c>
       <c r="J75" s="4" t="n">
-        <v>36.04</v>
+        <v>40.1</v>
       </c>
       <c r="K75" s="4" t="n">
-        <v>8.83</v>
+        <v>12.74</v>
       </c>
       <c r="L75" s="4" t="n">
-        <v>7.65</v>
+        <v>12.61</v>
       </c>
       <c r="M75" s="4" t="n">
-        <v>16.49</v>
+        <v>22.85</v>
       </c>
       <c r="N75" s="4" t="n">
-        <v>14.96</v>
+        <v>22.92</v>
       </c>
       <c r="O75" s="4" t="n">
-        <v>17.46</v>
+        <v>27.53</v>
       </c>
       <c r="P75" s="4" t="n">
-        <v>22.17</v>
+        <v>37.49</v>
       </c>
       <c r="Q75" s="4" t="n">
-        <v>5.22</v>
+        <v>16.18</v>
       </c>
       <c r="R75" s="4" t="n">
-        <v>15.58</v>
+        <v>34.49</v>
       </c>
       <c r="S75" s="4" t="n">
-        <v>26.68</v>
+        <v>65.69</v>
+      </c>
+      <c r="T75" s="4" t="n">
+        <v>56.06</v>
       </c>
     </row>
     <row r="76">
@@ -6380,6 +6603,10 @@
       </c>
       <c r="S76" s="6">
         <f>SUM(S4:S75)</f>
+        <v/>
+      </c>
+      <c r="T76" s="6">
+        <f>SUM(T4:T75)</f>
         <v/>
       </c>
     </row>
@@ -6421,7 +6648,8 @@
       <c r="P79" s="35" t="n"/>
       <c r="Q79" s="35" t="n"/>
       <c r="R79" s="35" t="n"/>
-      <c r="S79" s="36" t="n"/>
+      <c r="S79" s="35" t="n"/>
+      <c r="T79" s="36" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="37" t="n"/>
@@ -6515,6 +6743,11 @@
           <t>Jun</t>
         </is>
       </c>
+      <c r="T80" s="9" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
@@ -6594,6 +6827,10 @@
         <f>S68+S69</f>
         <v/>
       </c>
+      <c r="T81" s="11">
+        <f>T68+T69</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
@@ -6673,6 +6910,10 @@
         <f>S41+S42</f>
         <v/>
       </c>
+      <c r="T82" s="11">
+        <f>T41+T42</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
@@ -6752,6 +6993,10 @@
         <f>S21</f>
         <v/>
       </c>
+      <c r="T83" s="11">
+        <f>T21</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
@@ -6831,6 +7076,10 @@
         <f>S73</f>
         <v/>
       </c>
+      <c r="T84" s="11">
+        <f>T73</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
@@ -6910,6 +7159,10 @@
         <f>S50+S51</f>
         <v/>
       </c>
+      <c r="T85" s="11">
+        <f>T50+T51</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
@@ -6989,6 +7242,10 @@
         <f>S19+S20</f>
         <v/>
       </c>
+      <c r="T86" s="11">
+        <f>T19+T20</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
@@ -7068,6 +7325,10 @@
         <f>S56</f>
         <v/>
       </c>
+      <c r="T87" s="11">
+        <f>T56</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
@@ -7147,6 +7408,10 @@
         <f>S9</f>
         <v/>
       </c>
+      <c r="T88" s="11">
+        <f>T9</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
@@ -7226,6 +7491,10 @@
         <f>S22</f>
         <v/>
       </c>
+      <c r="T89" s="11">
+        <f>T22</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
@@ -7305,6 +7574,10 @@
         <f>S54</f>
         <v/>
       </c>
+      <c r="T90" s="11">
+        <f>T54</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
@@ -7384,6 +7657,10 @@
         <f>S25+S26</f>
         <v/>
       </c>
+      <c r="T91" s="11">
+        <f>T25+T26</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
@@ -7463,6 +7740,10 @@
         <f>S72</f>
         <v/>
       </c>
+      <c r="T92" s="11">
+        <f>T72</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
@@ -7542,6 +7823,10 @@
         <f>S59+S60</f>
         <v/>
       </c>
+      <c r="T93" s="11">
+        <f>T59+T60</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
@@ -7621,6 +7906,10 @@
         <f>+S95-SUM(S81:S93)</f>
         <v/>
       </c>
+      <c r="T94" s="11">
+        <f>+T95-SUM(T81:T93)</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="12" t="inlineStr">
@@ -7698,6 +7987,10 @@
       </c>
       <c r="S95" s="13">
         <f>+S76</f>
+        <v/>
+      </c>
+      <c r="T95" s="13">
+        <f>+T76</f>
         <v/>
       </c>
     </row>
@@ -8271,11 +8564,11 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="B2:M2"/>
-    <mergeCell ref="N2:S2"/>
     <mergeCell ref="A79:A80"/>
+    <mergeCell ref="N79:T79"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B79:M79"/>
-    <mergeCell ref="N79:S79"/>
+    <mergeCell ref="N2:T2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8289,13 +8582,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:S59"/>
+  <dimension ref="A3:T59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="47.140625" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="12.7109375" customWidth="1" min="2" max="19"/>
     <col width="13" customWidth="1" min="18" max="18"/>
     <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -8329,7 +8623,8 @@
       <c r="P3" s="35" t="n"/>
       <c r="Q3" s="35" t="n"/>
       <c r="R3" s="35" t="n"/>
-      <c r="S3" s="36" t="n"/>
+      <c r="S3" s="35" t="n"/>
+      <c r="T3" s="36" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="37" t="n"/>
@@ -8423,6 +8718,11 @@
           <t>Jun</t>
         </is>
       </c>
+      <c r="T4" s="26" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -8482,7 +8782,10 @@
         <v>96.43000000000001</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>109.95</v>
+        <v>133.4</v>
+      </c>
+      <c r="T5" s="4" t="n">
+        <v>143.37</v>
       </c>
     </row>
     <row r="6">
@@ -8543,7 +8846,10 @@
         <v>20.1</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>54.58</v>
+        <v>82.34</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>62.19</v>
       </c>
     </row>
     <row r="7">
@@ -8606,6 +8912,9 @@
       <c r="S7" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="T7" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -8667,6 +8976,9 @@
       <c r="S8" s="4" t="n">
         <v>2.19</v>
       </c>
+      <c r="T8" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -8728,6 +9040,9 @@
       <c r="S9" s="4" t="n">
         <v>73.15000000000001</v>
       </c>
+      <c r="T9" s="4" t="n">
+        <v>80.27</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -8789,6 +9104,9 @@
       <c r="S10" s="4" t="n">
         <v>69.90000000000001</v>
       </c>
+      <c r="T10" s="4" t="n">
+        <v>77.83</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -8850,6 +9168,9 @@
       <c r="S11" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="T11" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -8911,6 +9232,9 @@
       <c r="S12" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="T12" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -8972,6 +9296,9 @@
       <c r="S13" s="4" t="n">
         <v>128.39</v>
       </c>
+      <c r="T13" s="4" t="n">
+        <v>134.68</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -9031,7 +9358,10 @@
         <v>116.2</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>182.72</v>
+        <v>187.48</v>
+      </c>
+      <c r="T14" s="4" t="n">
+        <v>194.68</v>
       </c>
     </row>
     <row r="15">
@@ -9092,7 +9422,10 @@
         <v>84.84999999999999</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>128.79</v>
+        <v>133.96</v>
+      </c>
+      <c r="T15" s="4" t="n">
+        <v>84.5</v>
       </c>
     </row>
     <row r="16">
@@ -9153,7 +9486,10 @@
         <v>20.09</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>10.6</v>
+        <v>14.16</v>
+      </c>
+      <c r="T16" s="4" t="n">
+        <v>18.58</v>
       </c>
     </row>
     <row r="17">
@@ -9216,6 +9552,9 @@
       <c r="S17" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="T17" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -9275,7 +9614,10 @@
         <v>190.05</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>246.89</v>
+        <v>248.65</v>
+      </c>
+      <c r="T18" s="4" t="n">
+        <v>168.38</v>
       </c>
     </row>
     <row r="19">
@@ -9333,11 +9675,14 @@
         <v>64.04000000000001</v>
       </c>
       <c r="R19" s="4" t="n">
-        <v>35.06</v>
+        <v>35.51</v>
       </c>
       <c r="S19" s="4" t="n">
         <v>17.38</v>
       </c>
+      <c r="T19" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -9399,6 +9744,9 @@
       <c r="S20" s="4" t="n">
         <v>114.79</v>
       </c>
+      <c r="T20" s="4" t="n">
+        <v>50.33</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
@@ -9478,6 +9826,10 @@
         <f>SUM(S5:S20)</f>
         <v/>
       </c>
+      <c r="T21" s="28">
+        <f>SUM(T5:T20)</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="17.25" customHeight="1">
       <c r="A24" s="29" t="inlineStr">
@@ -9594,6 +9946,11 @@
           <t>Jun</t>
         </is>
       </c>
+      <c r="T26" s="31" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -9673,6 +10030,10 @@
         <f>S17+S18</f>
         <v/>
       </c>
+      <c r="T27" s="4">
+        <f>T17+T18</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -9752,6 +10113,10 @@
         <f>S11+S12</f>
         <v/>
       </c>
+      <c r="T28" s="4">
+        <f>T11+T12</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -9831,6 +10196,10 @@
         <f>S7</f>
         <v/>
       </c>
+      <c r="T29" s="4">
+        <f>T7</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -9910,6 +10279,10 @@
         <f>S19</f>
         <v/>
       </c>
+      <c r="T30" s="4">
+        <f>T19</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -9989,6 +10362,10 @@
         <f>S13+S14</f>
         <v/>
       </c>
+      <c r="T31" s="4">
+        <f>T13+T14</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -10068,6 +10445,10 @@
         <f>S9+S10</f>
         <v/>
       </c>
+      <c r="T32" s="4">
+        <f>T9+T10</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -10147,6 +10528,10 @@
         <f>S20</f>
         <v/>
       </c>
+      <c r="T33" s="4">
+        <f>T20</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -10226,6 +10611,10 @@
         <f>S6</f>
         <v/>
       </c>
+      <c r="T34" s="4">
+        <f>T6</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -10305,6 +10694,10 @@
         <f>S15</f>
         <v/>
       </c>
+      <c r="T35" s="4">
+        <f>T15</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -10384,6 +10777,10 @@
         <f>S5</f>
         <v/>
       </c>
+      <c r="T36" s="4">
+        <f>T5</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -10463,6 +10860,10 @@
         <f>S21-SUM(S27:S36)</f>
         <v/>
       </c>
+      <c r="T37" s="4">
+        <f>T21-SUM(T27:T36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
@@ -10540,6 +10941,10 @@
       </c>
       <c r="S38" s="28">
         <f>SUM(S27:S37)</f>
+        <v/>
+      </c>
+      <c r="T38" s="28">
+        <f>SUM(T27:T37)</f>
         <v/>
       </c>
     </row>
@@ -10995,11 +11400,11 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="B25:M25"/>
-    <mergeCell ref="N25:S25"/>
     <mergeCell ref="B3:M3"/>
     <mergeCell ref="A25:A26"/>
     <mergeCell ref="A3:A4"/>
-    <mergeCell ref="N3:S3"/>
+    <mergeCell ref="N3:T3"/>
+    <mergeCell ref="N25:T25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>